<commit_message>
docs: add TOTP authentication to INTEGRA MVP ERD and task plan
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KLewZ4X8CBFpmd4UfX8gco
</commit_message>
<xml_diff>
--- a/docs/Task_INTEGRA_MVP.xlsx
+++ b/docs/Task_INTEGRA_MVP.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Task" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Task'!$A$1:$L$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Task'!$A$1:$L$31</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -545,7 +545,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -677,19 +677,19 @@
         <v/>
       </c>
       <c r="B12" s="10">
-        <f>SUMIFS(Task!$I$2:$I$27,Task!$D$2:$D$27,A12,Task!$J$2:$J$27,"Hari 1")</f>
+        <f>SUMIFS(Task!$I$2:$I$31,Task!$D$2:$D$31,A12,Task!$J$2:$J$31,"Hari 1")</f>
         <v/>
       </c>
       <c r="C12" s="10">
-        <f>SUMIFS(Task!$I$2:$I$27,Task!$D$2:$D$27,A12,Task!$J$2:$J$27,"Hari 2")</f>
+        <f>SUMIFS(Task!$I$2:$I$31,Task!$D$2:$D$31,A12,Task!$J$2:$J$31,"Hari 2")</f>
         <v/>
       </c>
       <c r="D12" s="10">
-        <f>SUMIFS(Task!$I$2:$I$27,Task!$D$2:$D$27,A12,Task!$E$2:$E$27,"P0")</f>
+        <f>SUMIFS(Task!$I$2:$I$31,Task!$D$2:$D$31,A12,Task!$E$2:$E$31,"P0")</f>
         <v/>
       </c>
       <c r="E12" s="10">
-        <f>SUMIFS(Task!$I$2:$I$27,Task!$D$2:$D$27,A12,Task!$E$2:$E$27,"P1")</f>
+        <f>SUMIFS(Task!$I$2:$I$31,Task!$D$2:$D$31,A12,Task!$E$2:$E$31,"P1")</f>
         <v/>
       </c>
       <c r="F12" s="10">
@@ -697,7 +697,7 @@
         <v/>
       </c>
       <c r="G12" s="11">
-        <f>COUNTIFS(Task!$D$2:$D$27,A12,Task!$L$2:$L$27,"Selesai")</f>
+        <f>COUNTIFS(Task!$D$2:$D$31,A12,Task!$L$2:$L$31,"Selesai")</f>
         <v/>
       </c>
     </row>
@@ -707,19 +707,19 @@
         <v/>
       </c>
       <c r="B13" s="10">
-        <f>SUMIFS(Task!$I$2:$I$27,Task!$D$2:$D$27,A13,Task!$J$2:$J$27,"Hari 1")</f>
+        <f>SUMIFS(Task!$I$2:$I$31,Task!$D$2:$D$31,A13,Task!$J$2:$J$31,"Hari 1")</f>
         <v/>
       </c>
       <c r="C13" s="10">
-        <f>SUMIFS(Task!$I$2:$I$27,Task!$D$2:$D$27,A13,Task!$J$2:$J$27,"Hari 2")</f>
+        <f>SUMIFS(Task!$I$2:$I$31,Task!$D$2:$D$31,A13,Task!$J$2:$J$31,"Hari 2")</f>
         <v/>
       </c>
       <c r="D13" s="10">
-        <f>SUMIFS(Task!$I$2:$I$27,Task!$D$2:$D$27,A13,Task!$E$2:$E$27,"P0")</f>
+        <f>SUMIFS(Task!$I$2:$I$31,Task!$D$2:$D$31,A13,Task!$E$2:$E$31,"P0")</f>
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Task!$I$2:$I$27,Task!$D$2:$D$27,A13,Task!$E$2:$E$27,"P1")</f>
+        <f>SUMIFS(Task!$I$2:$I$31,Task!$D$2:$D$31,A13,Task!$E$2:$E$31,"P1")</f>
         <v/>
       </c>
       <c r="F13" s="10">
@@ -727,7 +727,7 @@
         <v/>
       </c>
       <c r="G13" s="11">
-        <f>COUNTIFS(Task!$D$2:$D$27,A13,Task!$L$2:$L$27,"Selesai")</f>
+        <f>COUNTIFS(Task!$D$2:$D$31,A13,Task!$L$2:$L$31,"Selesai")</f>
         <v/>
       </c>
     </row>
@@ -825,27 +825,27 @@
         </is>
       </c>
       <c r="B19" s="9">
-        <f>INDEX(Modul!$B$2:$B$11,MATCH(A19,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$B$2:$B$12,MATCH(A19,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="C19" s="11">
-        <f>INDEX(Modul!$C$2:$C$11,MATCH(A19,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$C$2:$C$12,MATCH(A19,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="D19" s="11">
-        <f>INDEX(Modul!$D$2:$D$11,MATCH(A19,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$D$2:$D$12,MATCH(A19,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="E19" s="11">
-        <f>COUNTIF(Task!$B$2:$B$27,A19)</f>
+        <f>COUNTIF(Task!$B$2:$B$31,A19)</f>
         <v/>
       </c>
       <c r="F19" s="10">
-        <f>SUMIF(Task!$B$2:$B$27,A19,Task!$I$2:$I$27)</f>
+        <f>SUMIF(Task!$B$2:$B$31,A19,Task!$I$2:$I$31)</f>
         <v/>
       </c>
       <c r="G19" s="11">
-        <f>COUNTIFS(Task!$B$2:$B$27,A19,Task!$L$2:$L$27,"Selesai")</f>
+        <f>COUNTIFS(Task!$B$2:$B$31,A19,Task!$L$2:$L$31,"Selesai")</f>
         <v/>
       </c>
       <c r="H19" s="15">
@@ -860,27 +860,27 @@
         </is>
       </c>
       <c r="B20" s="9">
-        <f>INDEX(Modul!$B$2:$B$11,MATCH(A20,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$B$2:$B$12,MATCH(A20,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="C20" s="11">
-        <f>INDEX(Modul!$C$2:$C$11,MATCH(A20,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$C$2:$C$12,MATCH(A20,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="D20" s="11">
-        <f>INDEX(Modul!$D$2:$D$11,MATCH(A20,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$D$2:$D$12,MATCH(A20,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="E20" s="11">
-        <f>COUNTIF(Task!$B$2:$B$27,A20)</f>
+        <f>COUNTIF(Task!$B$2:$B$31,A20)</f>
         <v/>
       </c>
       <c r="F20" s="10">
-        <f>SUMIF(Task!$B$2:$B$27,A20,Task!$I$2:$I$27)</f>
+        <f>SUMIF(Task!$B$2:$B$31,A20,Task!$I$2:$I$31)</f>
         <v/>
       </c>
       <c r="G20" s="11">
-        <f>COUNTIFS(Task!$B$2:$B$27,A20,Task!$L$2:$L$27,"Selesai")</f>
+        <f>COUNTIFS(Task!$B$2:$B$31,A20,Task!$L$2:$L$31,"Selesai")</f>
         <v/>
       </c>
       <c r="H20" s="15">
@@ -895,27 +895,27 @@
         </is>
       </c>
       <c r="B21" s="9">
-        <f>INDEX(Modul!$B$2:$B$11,MATCH(A21,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$B$2:$B$12,MATCH(A21,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="C21" s="11">
-        <f>INDEX(Modul!$C$2:$C$11,MATCH(A21,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$C$2:$C$12,MATCH(A21,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="D21" s="11">
-        <f>INDEX(Modul!$D$2:$D$11,MATCH(A21,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$D$2:$D$12,MATCH(A21,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="E21" s="11">
-        <f>COUNTIF(Task!$B$2:$B$27,A21)</f>
+        <f>COUNTIF(Task!$B$2:$B$31,A21)</f>
         <v/>
       </c>
       <c r="F21" s="10">
-        <f>SUMIF(Task!$B$2:$B$27,A21,Task!$I$2:$I$27)</f>
+        <f>SUMIF(Task!$B$2:$B$31,A21,Task!$I$2:$I$31)</f>
         <v/>
       </c>
       <c r="G21" s="11">
-        <f>COUNTIFS(Task!$B$2:$B$27,A21,Task!$L$2:$L$27,"Selesai")</f>
+        <f>COUNTIFS(Task!$B$2:$B$31,A21,Task!$L$2:$L$31,"Selesai")</f>
         <v/>
       </c>
       <c r="H21" s="15">
@@ -930,27 +930,27 @@
         </is>
       </c>
       <c r="B22" s="9">
-        <f>INDEX(Modul!$B$2:$B$11,MATCH(A22,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$B$2:$B$12,MATCH(A22,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="C22" s="11">
-        <f>INDEX(Modul!$C$2:$C$11,MATCH(A22,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$C$2:$C$12,MATCH(A22,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="D22" s="11">
-        <f>INDEX(Modul!$D$2:$D$11,MATCH(A22,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$D$2:$D$12,MATCH(A22,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="E22" s="11">
-        <f>COUNTIF(Task!$B$2:$B$27,A22)</f>
+        <f>COUNTIF(Task!$B$2:$B$31,A22)</f>
         <v/>
       </c>
       <c r="F22" s="10">
-        <f>SUMIF(Task!$B$2:$B$27,A22,Task!$I$2:$I$27)</f>
+        <f>SUMIF(Task!$B$2:$B$31,A22,Task!$I$2:$I$31)</f>
         <v/>
       </c>
       <c r="G22" s="11">
-        <f>COUNTIFS(Task!$B$2:$B$27,A22,Task!$L$2:$L$27,"Selesai")</f>
+        <f>COUNTIFS(Task!$B$2:$B$31,A22,Task!$L$2:$L$31,"Selesai")</f>
         <v/>
       </c>
       <c r="H22" s="15">
@@ -965,27 +965,27 @@
         </is>
       </c>
       <c r="B23" s="9">
-        <f>INDEX(Modul!$B$2:$B$11,MATCH(A23,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$B$2:$B$12,MATCH(A23,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="C23" s="11">
-        <f>INDEX(Modul!$C$2:$C$11,MATCH(A23,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$C$2:$C$12,MATCH(A23,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="D23" s="11">
-        <f>INDEX(Modul!$D$2:$D$11,MATCH(A23,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$D$2:$D$12,MATCH(A23,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="E23" s="11">
-        <f>COUNTIF(Task!$B$2:$B$27,A23)</f>
+        <f>COUNTIF(Task!$B$2:$B$31,A23)</f>
         <v/>
       </c>
       <c r="F23" s="10">
-        <f>SUMIF(Task!$B$2:$B$27,A23,Task!$I$2:$I$27)</f>
+        <f>SUMIF(Task!$B$2:$B$31,A23,Task!$I$2:$I$31)</f>
         <v/>
       </c>
       <c r="G23" s="11">
-        <f>COUNTIFS(Task!$B$2:$B$27,A23,Task!$L$2:$L$27,"Selesai")</f>
+        <f>COUNTIFS(Task!$B$2:$B$31,A23,Task!$L$2:$L$31,"Selesai")</f>
         <v/>
       </c>
       <c r="H23" s="15">
@@ -1000,27 +1000,27 @@
         </is>
       </c>
       <c r="B24" s="9">
-        <f>INDEX(Modul!$B$2:$B$11,MATCH(A24,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$B$2:$B$12,MATCH(A24,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="C24" s="11">
-        <f>INDEX(Modul!$C$2:$C$11,MATCH(A24,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$C$2:$C$12,MATCH(A24,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="D24" s="11">
-        <f>INDEX(Modul!$D$2:$D$11,MATCH(A24,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$D$2:$D$12,MATCH(A24,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="E24" s="11">
-        <f>COUNTIF(Task!$B$2:$B$27,A24)</f>
+        <f>COUNTIF(Task!$B$2:$B$31,A24)</f>
         <v/>
       </c>
       <c r="F24" s="10">
-        <f>SUMIF(Task!$B$2:$B$27,A24,Task!$I$2:$I$27)</f>
+        <f>SUMIF(Task!$B$2:$B$31,A24,Task!$I$2:$I$31)</f>
         <v/>
       </c>
       <c r="G24" s="11">
-        <f>COUNTIFS(Task!$B$2:$B$27,A24,Task!$L$2:$L$27,"Selesai")</f>
+        <f>COUNTIFS(Task!$B$2:$B$31,A24,Task!$L$2:$L$31,"Selesai")</f>
         <v/>
       </c>
       <c r="H24" s="15">
@@ -1035,27 +1035,27 @@
         </is>
       </c>
       <c r="B25" s="9">
-        <f>INDEX(Modul!$B$2:$B$11,MATCH(A25,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$B$2:$B$12,MATCH(A25,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="C25" s="11">
-        <f>INDEX(Modul!$C$2:$C$11,MATCH(A25,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$C$2:$C$12,MATCH(A25,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="D25" s="11">
-        <f>INDEX(Modul!$D$2:$D$11,MATCH(A25,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$D$2:$D$12,MATCH(A25,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="E25" s="11">
-        <f>COUNTIF(Task!$B$2:$B$27,A25)</f>
+        <f>COUNTIF(Task!$B$2:$B$31,A25)</f>
         <v/>
       </c>
       <c r="F25" s="10">
-        <f>SUMIF(Task!$B$2:$B$27,A25,Task!$I$2:$I$27)</f>
+        <f>SUMIF(Task!$B$2:$B$31,A25,Task!$I$2:$I$31)</f>
         <v/>
       </c>
       <c r="G25" s="11">
-        <f>COUNTIFS(Task!$B$2:$B$27,A25,Task!$L$2:$L$27,"Selesai")</f>
+        <f>COUNTIFS(Task!$B$2:$B$31,A25,Task!$L$2:$L$31,"Selesai")</f>
         <v/>
       </c>
       <c r="H25" s="15">
@@ -1070,27 +1070,27 @@
         </is>
       </c>
       <c r="B26" s="9">
-        <f>INDEX(Modul!$B$2:$B$11,MATCH(A26,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$B$2:$B$12,MATCH(A26,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="C26" s="11">
-        <f>INDEX(Modul!$C$2:$C$11,MATCH(A26,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$C$2:$C$12,MATCH(A26,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="D26" s="11">
-        <f>INDEX(Modul!$D$2:$D$11,MATCH(A26,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$D$2:$D$12,MATCH(A26,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="E26" s="11">
-        <f>COUNTIF(Task!$B$2:$B$27,A26)</f>
+        <f>COUNTIF(Task!$B$2:$B$31,A26)</f>
         <v/>
       </c>
       <c r="F26" s="10">
-        <f>SUMIF(Task!$B$2:$B$27,A26,Task!$I$2:$I$27)</f>
+        <f>SUMIF(Task!$B$2:$B$31,A26,Task!$I$2:$I$31)</f>
         <v/>
       </c>
       <c r="G26" s="11">
-        <f>COUNTIFS(Task!$B$2:$B$27,A26,Task!$L$2:$L$27,"Selesai")</f>
+        <f>COUNTIFS(Task!$B$2:$B$31,A26,Task!$L$2:$L$31,"Selesai")</f>
         <v/>
       </c>
       <c r="H26" s="15">
@@ -1105,27 +1105,27 @@
         </is>
       </c>
       <c r="B27" s="9">
-        <f>INDEX(Modul!$B$2:$B$11,MATCH(A27,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$B$2:$B$12,MATCH(A27,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="C27" s="11">
-        <f>INDEX(Modul!$C$2:$C$11,MATCH(A27,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$C$2:$C$12,MATCH(A27,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="D27" s="11">
-        <f>INDEX(Modul!$D$2:$D$11,MATCH(A27,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$D$2:$D$12,MATCH(A27,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="E27" s="11">
-        <f>COUNTIF(Task!$B$2:$B$27,A27)</f>
+        <f>COUNTIF(Task!$B$2:$B$31,A27)</f>
         <v/>
       </c>
       <c r="F27" s="10">
-        <f>SUMIF(Task!$B$2:$B$27,A27,Task!$I$2:$I$27)</f>
+        <f>SUMIF(Task!$B$2:$B$31,A27,Task!$I$2:$I$31)</f>
         <v/>
       </c>
       <c r="G27" s="11">
-        <f>COUNTIFS(Task!$B$2:$B$27,A27,Task!$L$2:$L$27,"Selesai")</f>
+        <f>COUNTIFS(Task!$B$2:$B$31,A27,Task!$L$2:$L$31,"Selesai")</f>
         <v/>
       </c>
       <c r="H27" s="15">
@@ -1140,27 +1140,27 @@
         </is>
       </c>
       <c r="B28" s="9">
-        <f>INDEX(Modul!$B$2:$B$11,MATCH(A28,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$B$2:$B$12,MATCH(A28,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="C28" s="11">
-        <f>INDEX(Modul!$C$2:$C$11,MATCH(A28,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$C$2:$C$12,MATCH(A28,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="D28" s="11">
-        <f>INDEX(Modul!$D$2:$D$11,MATCH(A28,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$D$2:$D$12,MATCH(A28,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="E28" s="11">
-        <f>COUNTIF(Task!$B$2:$B$27,A28)</f>
+        <f>COUNTIF(Task!$B$2:$B$31,A28)</f>
         <v/>
       </c>
       <c r="F28" s="10">
-        <f>SUMIF(Task!$B$2:$B$27,A28,Task!$I$2:$I$27)</f>
+        <f>SUMIF(Task!$B$2:$B$31,A28,Task!$I$2:$I$31)</f>
         <v/>
       </c>
       <c r="G28" s="11">
-        <f>COUNTIFS(Task!$B$2:$B$27,A28,Task!$L$2:$L$27,"Selesai")</f>
+        <f>COUNTIFS(Task!$B$2:$B$31,A28,Task!$L$2:$L$31,"Selesai")</f>
         <v/>
       </c>
       <c r="H28" s="15">
@@ -1169,28 +1169,63 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="14" t="inlineStr">
+      <c r="A29" s="11" t="inlineStr">
+        <is>
+          <t>M-11</t>
+        </is>
+      </c>
+      <c r="B29" s="9">
+        <f>INDEX(Modul!$B$2:$B$12,MATCH(A29,Modul!$A$2:$A$12,0))</f>
+        <v/>
+      </c>
+      <c r="C29" s="11">
+        <f>INDEX(Modul!$C$2:$C$12,MATCH(A29,Modul!$A$2:$A$12,0))</f>
+        <v/>
+      </c>
+      <c r="D29" s="11">
+        <f>INDEX(Modul!$D$2:$D$12,MATCH(A29,Modul!$A$2:$A$12,0))</f>
+        <v/>
+      </c>
+      <c r="E29" s="11">
+        <f>COUNTIF(Task!$B$2:$B$31,A29)</f>
+        <v/>
+      </c>
+      <c r="F29" s="10">
+        <f>SUMIF(Task!$B$2:$B$31,A29,Task!$I$2:$I$31)</f>
+        <v/>
+      </c>
+      <c r="G29" s="11">
+        <f>COUNTIFS(Task!$B$2:$B$31,A29,Task!$L$2:$L$31,"Selesai")</f>
+        <v/>
+      </c>
+      <c r="H29" s="15">
+        <f>IF(E29=0,"-",G29/E29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="14" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B29" s="12" t="n"/>
-      <c r="C29" s="14" t="n"/>
-      <c r="D29" s="14" t="n"/>
-      <c r="E29" s="14">
-        <f>SUM(E19:E28)</f>
-        <v/>
-      </c>
-      <c r="F29" s="13">
-        <f>SUM(F19:F28)</f>
-        <v/>
-      </c>
-      <c r="G29" s="14">
-        <f>SUM(G19:G28)</f>
-        <v/>
-      </c>
-      <c r="H29" s="16">
-        <f>IF(E29=0,"-",G29/E29)</f>
+      <c r="B30" s="12" t="n"/>
+      <c r="C30" s="14" t="n"/>
+      <c r="D30" s="14" t="n"/>
+      <c r="E30" s="14">
+        <f>SUM(E19:E29)</f>
+        <v/>
+      </c>
+      <c r="F30" s="13">
+        <f>SUM(F19:F29)</f>
+        <v/>
+      </c>
+      <c r="G30" s="14">
+        <f>SUM(G19:G29)</f>
+        <v/>
+      </c>
+      <c r="H30" s="16">
+        <f>IF(E30=0,"-",G30/E30)</f>
         <v/>
       </c>
     </row>
@@ -1205,7 +1240,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1792,9 +1827,61 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>M-11</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Autentikasi TOTP</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D12" s="17" t="inlineStr">
+        <is>
+          <t>Orang B</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>Tata kelola: akses dibatasi per peran, keputusan tercatat</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>Login email + kode TOTP dari aplikasi authenticator, sesi JWT di cookie httpOnly, dan pembatasan akses per peran.</t>
+        </is>
+      </c>
+      <c r="G12" s="9" t="inlineStr">
+        <is>
+          <t>POST /auth/login, POST /auth/logout, GET /auth/me, guard JWT + peran</t>
+        </is>
+      </c>
+      <c r="H12" s="9" t="inlineStr">
+        <is>
+          <t>Halaman login, proteksi route</t>
+        </is>
+      </c>
+      <c r="I12" s="9" t="inlineStr">
+        <is>
+          <t>users</t>
+        </is>
+      </c>
+      <c r="J12" s="9" t="inlineStr">
+        <is>
+          <t>M-01</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="D2:D31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D2:D32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Orang A,Orang B"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1808,7 +1895,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1876,11 +1963,11 @@
         </is>
       </c>
       <c r="B2" s="9">
-        <f>INDEX(Modul!$B$2:$B$11,MATCH(A2,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$B$2:$B$12,MATCH(A2,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="C2" s="11">
-        <f>INDEX(Modul!$C$2:$C$11,MATCH(A2,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$C$2:$C$12,MATCH(A2,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="D2" s="9" t="inlineStr">
@@ -1899,12 +1986,13 @@
 - Migrasi dan PrismaModule
 - Repository Prisma
 - Kontrak JSON extracted dan response GET /claims/:id
+- Config env tervalidasi, exception filter, CORS
 - Layout dan navigasi web</t>
         </is>
       </c>
       <c r="G2" s="9" t="inlineStr">
         <is>
-          <t>- Autentikasi dan manajemen pengguna</t>
+          <t>- Autentikasi (ada di M-11)</t>
         </is>
       </c>
       <c r="H2" s="9" t="inlineStr">
@@ -1927,11 +2015,11 @@
         </is>
       </c>
       <c r="B3" s="9">
-        <f>INDEX(Modul!$B$2:$B$11,MATCH(A3,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$B$2:$B$12,MATCH(A3,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="C3" s="11">
-        <f>INDEX(Modul!$C$2:$C$11,MATCH(A3,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$C$2:$C$12,MATCH(A3,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="D3" s="9" t="inlineStr">
@@ -1978,11 +2066,11 @@
         </is>
       </c>
       <c r="B4" s="9">
-        <f>INDEX(Modul!$B$2:$B$11,MATCH(A4,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$B$2:$B$12,MATCH(A4,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="C4" s="11">
-        <f>INDEX(Modul!$C$2:$C$11,MATCH(A4,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$C$2:$C$12,MATCH(A4,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="D4" s="9" t="inlineStr">
@@ -2028,11 +2116,11 @@
         </is>
       </c>
       <c r="B5" s="9">
-        <f>INDEX(Modul!$B$2:$B$11,MATCH(A5,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$B$2:$B$12,MATCH(A5,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="C5" s="11">
-        <f>INDEX(Modul!$C$2:$C$11,MATCH(A5,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$C$2:$C$12,MATCH(A5,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="D5" s="9" t="inlineStr">
@@ -2077,11 +2165,11 @@
         </is>
       </c>
       <c r="B6" s="9">
-        <f>INDEX(Modul!$B$2:$B$11,MATCH(A6,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$B$2:$B$12,MATCH(A6,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="C6" s="11">
-        <f>INDEX(Modul!$C$2:$C$11,MATCH(A6,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$C$2:$C$12,MATCH(A6,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="D6" s="9" t="inlineStr">
@@ -2126,11 +2214,11 @@
         </is>
       </c>
       <c r="B7" s="9">
-        <f>INDEX(Modul!$B$2:$B$11,MATCH(A7,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$B$2:$B$12,MATCH(A7,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="C7" s="11">
-        <f>INDEX(Modul!$C$2:$C$11,MATCH(A7,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$C$2:$C$12,MATCH(A7,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="D7" s="9" t="inlineStr">
@@ -2176,11 +2264,11 @@
         </is>
       </c>
       <c r="B8" s="9">
-        <f>INDEX(Modul!$B$2:$B$11,MATCH(A8,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$B$2:$B$12,MATCH(A8,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="C8" s="11">
-        <f>INDEX(Modul!$C$2:$C$11,MATCH(A8,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$C$2:$C$12,MATCH(A8,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="D8" s="9" t="inlineStr">
@@ -2225,11 +2313,11 @@
         </is>
       </c>
       <c r="B9" s="9">
-        <f>INDEX(Modul!$B$2:$B$11,MATCH(A9,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$B$2:$B$12,MATCH(A9,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="C9" s="11">
-        <f>INDEX(Modul!$C$2:$C$11,MATCH(A9,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$C$2:$C$12,MATCH(A9,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="D9" s="9" t="inlineStr">
@@ -2272,11 +2360,11 @@
         </is>
       </c>
       <c r="B10" s="9">
-        <f>INDEX(Modul!$B$2:$B$11,MATCH(A10,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$B$2:$B$12,MATCH(A10,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="C10" s="11">
-        <f>INDEX(Modul!$C$2:$C$11,MATCH(A10,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$C$2:$C$12,MATCH(A10,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="D10" s="9" t="inlineStr">
@@ -2319,11 +2407,11 @@
         </is>
       </c>
       <c r="B11" s="9">
-        <f>INDEX(Modul!$B$2:$B$11,MATCH(A11,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$B$2:$B$12,MATCH(A11,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="C11" s="11">
-        <f>INDEX(Modul!$C$2:$C$11,MATCH(A11,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$C$2:$C$12,MATCH(A11,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="D11" s="9" t="inlineStr">
@@ -2354,6 +2442,57 @@
       <c r="I11" s="9" t="inlineStr">
         <is>
           <t>Persona supervisor</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>M-11</t>
+        </is>
+      </c>
+      <c r="B12" s="9">
+        <f>INDEX(Modul!$B$2:$B$12,MATCH(A12,Modul!$A$2:$A$12,0))</f>
+        <v/>
+      </c>
+      <c r="C12" s="11">
+        <f>INDEX(Modul!$C$2:$C$12,MATCH(A12,Modul!$A$2:$A$12,0))</f>
+        <v/>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>Hanya verifikator dan supervisor terdaftar yang bisa membuka antrean dan Kartu Klaim.</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>Sebagai verifikator, saya ingin login dengan kode authenticator supaya keputusan saya tercatat atas nama saya.</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>- Seed secret TOTP terenkripsi + script QR otpauth
+- Login email + kode 6 digit, anti-replay lewat totp_last_step
+- JWT di cookie httpOnly
+- Guard global, @Public untuk login dan health, @Roles untuk supervisor
+- Rate limit endpoint login</t>
+        </is>
+      </c>
+      <c r="G12" s="9" t="inlineStr">
+        <is>
+          <t>- Password, halaman enrolment, reset TOTP, manajemen pengguna</t>
+        </is>
+      </c>
+      <c r="H12" s="9" t="inlineStr">
+        <is>
+          <t>- Kode salah atau dipakai ulang ditolak
+- Endpoint klaim menolak request tanpa cookie
+- verifier_id di decisions diambil dari user login, bukan dari body</t>
+        </is>
+      </c>
+      <c r="I12" s="9" t="inlineStr">
+        <is>
+          <t>Tata kelola, privasi, dan risiko</t>
         </is>
       </c>
     </row>
@@ -2368,7 +2507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L27"/>
+  <dimension ref="A1:L31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2459,11 +2598,11 @@
         </is>
       </c>
       <c r="C2" s="9">
-        <f>INDEX(Modul!$B$2:$B$11,MATCH(B2,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$B$2:$B$12,MATCH(B2,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="D2" s="11">
-        <f>INDEX(Modul!$D$2:$D$11,MATCH(B2,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$D$2:$D$12,MATCH(B2,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="E2" s="11" t="inlineStr">
@@ -2517,11 +2656,11 @@
         </is>
       </c>
       <c r="C3" s="9">
-        <f>INDEX(Modul!$B$2:$B$11,MATCH(B3,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$B$2:$B$12,MATCH(B3,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="D3" s="11">
-        <f>INDEX(Modul!$D$2:$D$11,MATCH(B3,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$D$2:$D$12,MATCH(B3,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="E3" s="11" t="inlineStr">
@@ -2575,11 +2714,11 @@
         </is>
       </c>
       <c r="C4" s="9">
-        <f>INDEX(Modul!$B$2:$B$11,MATCH(B4,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$B$2:$B$12,MATCH(B4,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="D4" s="11">
-        <f>INDEX(Modul!$D$2:$D$11,MATCH(B4,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$D$2:$D$12,MATCH(B4,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="E4" s="11" t="inlineStr">
@@ -2633,11 +2772,11 @@
         </is>
       </c>
       <c r="C5" s="9">
-        <f>INDEX(Modul!$B$2:$B$11,MATCH(B5,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$B$2:$B$12,MATCH(B5,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="D5" s="11">
-        <f>INDEX(Modul!$D$2:$D$11,MATCH(B5,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$D$2:$D$12,MATCH(B5,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="E5" s="11" t="inlineStr">
@@ -2691,11 +2830,11 @@
         </is>
       </c>
       <c r="C6" s="9">
-        <f>INDEX(Modul!$B$2:$B$11,MATCH(B6,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$B$2:$B$12,MATCH(B6,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="D6" s="11">
-        <f>INDEX(Modul!$D$2:$D$11,MATCH(B6,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$D$2:$D$12,MATCH(B6,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="E6" s="11" t="inlineStr">
@@ -2749,11 +2888,11 @@
         </is>
       </c>
       <c r="C7" s="9">
-        <f>INDEX(Modul!$B$2:$B$11,MATCH(B7,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$B$2:$B$12,MATCH(B7,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="D7" s="11">
-        <f>INDEX(Modul!$D$2:$D$11,MATCH(B7,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$D$2:$D$12,MATCH(B7,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="E7" s="11" t="inlineStr">
@@ -2807,11 +2946,11 @@
         </is>
       </c>
       <c r="C8" s="9">
-        <f>INDEX(Modul!$B$2:$B$11,MATCH(B8,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$B$2:$B$12,MATCH(B8,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="D8" s="11">
-        <f>INDEX(Modul!$D$2:$D$11,MATCH(B8,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$D$2:$D$12,MATCH(B8,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="E8" s="11" t="inlineStr">
@@ -2865,11 +3004,11 @@
         </is>
       </c>
       <c r="C9" s="9">
-        <f>INDEX(Modul!$B$2:$B$11,MATCH(B9,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$B$2:$B$12,MATCH(B9,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="D9" s="11">
-        <f>INDEX(Modul!$D$2:$D$11,MATCH(B9,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$D$2:$D$12,MATCH(B9,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="E9" s="11" t="inlineStr">
@@ -2923,11 +3062,11 @@
         </is>
       </c>
       <c r="C10" s="9">
-        <f>INDEX(Modul!$B$2:$B$11,MATCH(B10,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$B$2:$B$12,MATCH(B10,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="D10" s="11">
-        <f>INDEX(Modul!$D$2:$D$11,MATCH(B10,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$D$2:$D$12,MATCH(B10,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="E10" s="11" t="inlineStr">
@@ -2981,11 +3120,11 @@
         </is>
       </c>
       <c r="C11" s="9">
-        <f>INDEX(Modul!$B$2:$B$11,MATCH(B11,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$B$2:$B$12,MATCH(B11,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="D11" s="11">
-        <f>INDEX(Modul!$D$2:$D$11,MATCH(B11,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$D$2:$D$12,MATCH(B11,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="E11" s="11" t="inlineStr">
@@ -3039,11 +3178,11 @@
         </is>
       </c>
       <c r="C12" s="9">
-        <f>INDEX(Modul!$B$2:$B$11,MATCH(B12,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$B$2:$B$12,MATCH(B12,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="D12" s="11">
-        <f>INDEX(Modul!$D$2:$D$11,MATCH(B12,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$D$2:$D$12,MATCH(B12,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="E12" s="11" t="inlineStr">
@@ -3097,11 +3236,11 @@
         </is>
       </c>
       <c r="C13" s="9">
-        <f>INDEX(Modul!$B$2:$B$11,MATCH(B13,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$B$2:$B$12,MATCH(B13,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="D13" s="11">
-        <f>INDEX(Modul!$D$2:$D$11,MATCH(B13,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$D$2:$D$12,MATCH(B13,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="E13" s="11" t="inlineStr">
@@ -3155,11 +3294,11 @@
         </is>
       </c>
       <c r="C14" s="9">
-        <f>INDEX(Modul!$B$2:$B$11,MATCH(B14,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$B$2:$B$12,MATCH(B14,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="D14" s="11">
-        <f>INDEX(Modul!$D$2:$D$11,MATCH(B14,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$D$2:$D$12,MATCH(B14,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="E14" s="11" t="inlineStr">
@@ -3213,11 +3352,11 @@
         </is>
       </c>
       <c r="C15" s="9">
-        <f>INDEX(Modul!$B$2:$B$11,MATCH(B15,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$B$2:$B$12,MATCH(B15,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="D15" s="11">
-        <f>INDEX(Modul!$D$2:$D$11,MATCH(B15,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$D$2:$D$12,MATCH(B15,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="E15" s="11" t="inlineStr">
@@ -3271,11 +3410,11 @@
         </is>
       </c>
       <c r="C16" s="9">
-        <f>INDEX(Modul!$B$2:$B$11,MATCH(B16,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$B$2:$B$12,MATCH(B16,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="D16" s="11">
-        <f>INDEX(Modul!$D$2:$D$11,MATCH(B16,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$D$2:$D$12,MATCH(B16,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="E16" s="11" t="inlineStr">
@@ -3329,11 +3468,11 @@
         </is>
       </c>
       <c r="C17" s="9">
-        <f>INDEX(Modul!$B$2:$B$11,MATCH(B17,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$B$2:$B$12,MATCH(B17,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="D17" s="11">
-        <f>INDEX(Modul!$D$2:$D$11,MATCH(B17,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$D$2:$D$12,MATCH(B17,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="E17" s="11" t="inlineStr">
@@ -3387,11 +3526,11 @@
         </is>
       </c>
       <c r="C18" s="9">
-        <f>INDEX(Modul!$B$2:$B$11,MATCH(B18,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$B$2:$B$12,MATCH(B18,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="D18" s="11">
-        <f>INDEX(Modul!$D$2:$D$11,MATCH(B18,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$D$2:$D$12,MATCH(B18,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="E18" s="11" t="inlineStr">
@@ -3445,11 +3584,11 @@
         </is>
       </c>
       <c r="C19" s="9">
-        <f>INDEX(Modul!$B$2:$B$11,MATCH(B19,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$B$2:$B$12,MATCH(B19,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="D19" s="11">
-        <f>INDEX(Modul!$D$2:$D$11,MATCH(B19,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$D$2:$D$12,MATCH(B19,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="E19" s="11" t="inlineStr">
@@ -3503,11 +3642,11 @@
         </is>
       </c>
       <c r="C20" s="9">
-        <f>INDEX(Modul!$B$2:$B$11,MATCH(B20,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$B$2:$B$12,MATCH(B20,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="D20" s="11">
-        <f>INDEX(Modul!$D$2:$D$11,MATCH(B20,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$D$2:$D$12,MATCH(B20,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="E20" s="11" t="inlineStr">
@@ -3561,11 +3700,11 @@
         </is>
       </c>
       <c r="C21" s="9">
-        <f>INDEX(Modul!$B$2:$B$11,MATCH(B21,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$B$2:$B$12,MATCH(B21,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="D21" s="11">
-        <f>INDEX(Modul!$D$2:$D$11,MATCH(B21,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$D$2:$D$12,MATCH(B21,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="E21" s="11" t="inlineStr">
@@ -3619,11 +3758,11 @@
         </is>
       </c>
       <c r="C22" s="9">
-        <f>INDEX(Modul!$B$2:$B$11,MATCH(B22,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$B$2:$B$12,MATCH(B22,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="D22" s="11">
-        <f>INDEX(Modul!$D$2:$D$11,MATCH(B22,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$D$2:$D$12,MATCH(B22,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="E22" s="11" t="inlineStr">
@@ -3677,11 +3816,11 @@
         </is>
       </c>
       <c r="C23" s="9">
-        <f>INDEX(Modul!$B$2:$B$11,MATCH(B23,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$B$2:$B$12,MATCH(B23,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="D23" s="11">
-        <f>INDEX(Modul!$D$2:$D$11,MATCH(B23,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$D$2:$D$12,MATCH(B23,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="E23" s="11" t="inlineStr">
@@ -3735,11 +3874,11 @@
         </is>
       </c>
       <c r="C24" s="9">
-        <f>INDEX(Modul!$B$2:$B$11,MATCH(B24,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$B$2:$B$12,MATCH(B24,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="D24" s="11">
-        <f>INDEX(Modul!$D$2:$D$11,MATCH(B24,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$D$2:$D$12,MATCH(B24,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="E24" s="11" t="inlineStr">
@@ -3793,11 +3932,11 @@
         </is>
       </c>
       <c r="C25" s="9">
-        <f>INDEX(Modul!$B$2:$B$11,MATCH(B25,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$B$2:$B$12,MATCH(B25,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="D25" s="11">
-        <f>INDEX(Modul!$D$2:$D$11,MATCH(B25,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$D$2:$D$12,MATCH(B25,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="E25" s="11" t="inlineStr">
@@ -3851,11 +3990,11 @@
         </is>
       </c>
       <c r="C26" s="9">
-        <f>INDEX(Modul!$B$2:$B$11,MATCH(B26,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$B$2:$B$12,MATCH(B26,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="D26" s="11">
-        <f>INDEX(Modul!$D$2:$D$11,MATCH(B26,Modul!$A$2:$A$11,0))</f>
+        <f>INDEX(Modul!$D$2:$D$12,MATCH(B26,Modul!$A$2:$A$12,0))</f>
         <v/>
       </c>
       <c r="E26" s="11" t="inlineStr">
@@ -3900,64 +4039,296 @@
     <row r="27">
       <c r="A27" s="11" t="inlineStr">
         <is>
+          <t>T27</t>
+        </is>
+      </c>
+      <c r="B27" s="11" t="inlineStr">
+        <is>
+          <t>M-01</t>
+        </is>
+      </c>
+      <c r="C27" s="9">
+        <f>INDEX(Modul!$B$2:$B$12,MATCH(B27,Modul!$A$2:$A$12,0))</f>
+        <v/>
+      </c>
+      <c r="D27" s="11">
+        <f>INDEX(Modul!$D$2:$D$12,MATCH(B27,Modul!$A$2:$A$12,0))</f>
+        <v/>
+      </c>
+      <c r="E27" s="11" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="F27" s="9" t="inlineStr">
+        <is>
+          <t>Config dan HTTP lintas modul</t>
+        </is>
+      </c>
+      <c r="G27" s="9" t="inlineStr">
+        <is>
+          <t>ConfigModule dengan validasi env, exception filter domain error ke HTTP, CORS dengan credentials, cookie-parser</t>
+        </is>
+      </c>
+      <c r="H27" s="11" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="I27" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="J27" s="11" t="inlineStr">
+        <is>
+          <t>Hari 1</t>
+        </is>
+      </c>
+      <c r="K27" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L27" s="17" t="inlineStr">
+        <is>
+          <t>Belum mulai</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="11" t="inlineStr">
+        <is>
+          <t>T28</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>M-11</t>
+        </is>
+      </c>
+      <c r="C28" s="9">
+        <f>INDEX(Modul!$B$2:$B$12,MATCH(B28,Modul!$A$2:$A$12,0))</f>
+        <v/>
+      </c>
+      <c r="D28" s="11">
+        <f>INDEX(Modul!$D$2:$D$12,MATCH(B28,Modul!$A$2:$A$12,0))</f>
+        <v/>
+      </c>
+      <c r="E28" s="11" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="F28" s="9" t="inlineStr">
+        <is>
+          <t>Seed secret TOTP dan QR</t>
+        </is>
+      </c>
+      <c r="G28" s="9" t="inlineStr">
+        <is>
+          <t>Generate secret per user, simpan terenkripsi AES-256-GCM, cetak QR otpauth untuk dipindai</t>
+        </is>
+      </c>
+      <c r="H28" s="11" t="inlineStr">
+        <is>
+          <t>Database</t>
+        </is>
+      </c>
+      <c r="I28" s="18" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J28" s="11" t="inlineStr">
+        <is>
+          <t>Hari 1</t>
+        </is>
+      </c>
+      <c r="K28" s="9" t="inlineStr">
+        <is>
+          <t>T07</t>
+        </is>
+      </c>
+      <c r="L28" s="17" t="inlineStr">
+        <is>
+          <t>Belum mulai</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="11" t="inlineStr">
+        <is>
+          <t>T29</t>
+        </is>
+      </c>
+      <c r="B29" s="11" t="inlineStr">
+        <is>
+          <t>M-11</t>
+        </is>
+      </c>
+      <c r="C29" s="9">
+        <f>INDEX(Modul!$B$2:$B$12,MATCH(B29,Modul!$A$2:$A$12,0))</f>
+        <v/>
+      </c>
+      <c r="D29" s="11">
+        <f>INDEX(Modul!$D$2:$D$12,MATCH(B29,Modul!$A$2:$A$12,0))</f>
+        <v/>
+      </c>
+      <c r="E29" s="11" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="F29" s="9" t="inlineStr">
+        <is>
+          <t>API autentikasi TOTP</t>
+        </is>
+      </c>
+      <c r="G29" s="9" t="inlineStr">
+        <is>
+          <t>Use case login (verifikasi kode, cek totp_last_step), JWT cookie httpOnly, /auth/me, /auth/logout, guard global + @Public + @Roles, throttler</t>
+        </is>
+      </c>
+      <c r="H29" s="11" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="I29" s="18" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="J29" s="11" t="inlineStr">
+        <is>
+          <t>Hari 2</t>
+        </is>
+      </c>
+      <c r="K29" s="9" t="inlineStr">
+        <is>
+          <t>T27, T28</t>
+        </is>
+      </c>
+      <c r="L29" s="17" t="inlineStr">
+        <is>
+          <t>Belum mulai</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="11" t="inlineStr">
+        <is>
+          <t>T30</t>
+        </is>
+      </c>
+      <c r="B30" s="11" t="inlineStr">
+        <is>
+          <t>M-11</t>
+        </is>
+      </c>
+      <c r="C30" s="9">
+        <f>INDEX(Modul!$B$2:$B$12,MATCH(B30,Modul!$A$2:$A$12,0))</f>
+        <v/>
+      </c>
+      <c r="D30" s="11">
+        <f>INDEX(Modul!$D$2:$D$12,MATCH(B30,Modul!$A$2:$A$12,0))</f>
+        <v/>
+      </c>
+      <c r="E30" s="11" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="F30" s="9" t="inlineStr">
+        <is>
+          <t>Halaman login dan proteksi route</t>
+        </is>
+      </c>
+      <c r="G30" s="9" t="inlineStr">
+        <is>
+          <t>Form email + kode 6 digit, redirect ke login saat 401, tombol logout</t>
+        </is>
+      </c>
+      <c r="H30" s="11" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="I30" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="J30" s="11" t="inlineStr">
+        <is>
+          <t>Hari 2</t>
+        </is>
+      </c>
+      <c r="K30" s="9" t="inlineStr">
+        <is>
+          <t>T04, T29</t>
+        </is>
+      </c>
+      <c r="L30" s="17" t="inlineStr">
+        <is>
+          <t>Belum mulai</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="11" t="inlineStr">
+        <is>
           <t>T26</t>
         </is>
       </c>
-      <c r="B27" s="11" t="inlineStr">
+      <c r="B31" s="11" t="inlineStr">
         <is>
           <t>M-10</t>
         </is>
       </c>
-      <c r="C27" s="9">
-        <f>INDEX(Modul!$B$2:$B$11,MATCH(B27,Modul!$A$2:$A$11,0))</f>
-        <v/>
-      </c>
-      <c r="D27" s="11">
-        <f>INDEX(Modul!$D$2:$D$11,MATCH(B27,Modul!$A$2:$A$11,0))</f>
-        <v/>
-      </c>
-      <c r="E27" s="11" t="inlineStr">
+      <c r="C31" s="9">
+        <f>INDEX(Modul!$B$2:$B$12,MATCH(B31,Modul!$A$2:$A$12,0))</f>
+        <v/>
+      </c>
+      <c r="D31" s="11">
+        <f>INDEX(Modul!$D$2:$D$12,MATCH(B31,Modul!$A$2:$A$12,0))</f>
+        <v/>
+      </c>
+      <c r="E31" s="11" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F27" s="9" t="inlineStr">
+      <c r="F31" s="9" t="inlineStr">
         <is>
           <t>Ringkasan faskes</t>
         </is>
       </c>
-      <c r="G27" s="9" t="inlineStr">
+      <c r="G31" s="9" t="inlineStr">
         <is>
           <t>Endpoint agregat per faskes dan halaman ringkasan</t>
         </is>
       </c>
-      <c r="H27" s="11" t="inlineStr">
+      <c r="H31" s="11" t="inlineStr">
         <is>
           <t>API + Web</t>
         </is>
       </c>
-      <c r="I27" s="18" t="n">
+      <c r="I31" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="J27" s="11" t="inlineStr">
+      <c r="J31" s="11" t="inlineStr">
         <is>
           <t>Hari 2</t>
         </is>
       </c>
-      <c r="K27" s="9" t="inlineStr">
+      <c r="K31" s="9" t="inlineStr">
         <is>
           <t>T21</t>
         </is>
       </c>
-      <c r="L27" s="17" t="inlineStr">
+      <c r="L31" s="17" t="inlineStr">
         <is>
           <t>Belum mulai</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L27"/>
-  <conditionalFormatting sqref="A2:L27">
+  <autoFilter ref="A1:L31"/>
+  <conditionalFormatting sqref="A2:L31">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$L2="Selesai"</formula>
     </cfRule>
@@ -3966,20 +4337,20 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="5">
-    <dataValidation sqref="L2:L77" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="L2:L81" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Belum mulai,Dikerjakan,Selesai,Terblokir"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J77" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J81" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Hari 1,Hari 2"</formula1>
     </dataValidation>
-    <dataValidation sqref="H2:H77" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H2:H81" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Kontrak,Database,API,Web,API + Web,LLM,Data"</formula1>
     </dataValidation>
-    <dataValidation sqref="E2:E77" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E81" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"P0,P1"</formula1>
     </dataValidation>
-    <dataValidation sqref="B2:B77" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>=Modul!$A$2:$A$11</formula1>
+    <dataValidation sqref="B2:B81" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>=Modul!$A$2:$A$12</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>